<commit_message>
feat: add to graph the Enumerations as xlsx.
</commit_message>
<xml_diff>
--- a/plc/s7-1x00/core/adt/EAdtConstants-v1.1.xlsx
+++ b/plc/s7-1x00/core/adt/EAdtConstants-v1.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PlcFramework\code\plc\s7-1x00\core\adt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53B75E4B-1DF2-4B49-9635-58A0A6A4D453}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D9CC24D-4336-4D3B-88C0-ACD7F82D2078}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-10230" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Constants" sheetId="1" r:id="rId1"/>
@@ -498,14 +498,14 @@
     <t>Bool</t>
   </si>
   <si>
-    <t>{"version":"v1.0","author":"cyanezf","family":"core/adt"}</t>
+    <t>{"version":"v1.1","author":"cyanezf","family":"core/adt","status":"current","deprecatedBy":null,"dependencies":[]}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -876,16 +876,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E66"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="50.453125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.90625" customWidth="1"/>
     <col min="3" max="3" width="9.7265625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="57.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="101.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -902,7 +902,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>152</v>
       </c>
@@ -919,7 +919,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -936,7 +936,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -953,7 +953,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -970,7 +970,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -987,7 +987,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>23</v>
       </c>
@@ -1004,7 +1004,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>26</v>
       </c>
@@ -1021,7 +1021,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>29</v>
       </c>
@@ -1038,7 +1038,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>32</v>
       </c>
@@ -1055,7 +1055,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>35</v>
       </c>
@@ -1072,7 +1072,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -1089,7 +1089,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>41</v>
       </c>
@@ -1106,7 +1106,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>44</v>
       </c>
@@ -1123,7 +1123,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>47</v>
       </c>
@@ -1140,7 +1140,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>50</v>
       </c>
@@ -1157,7 +1157,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>53</v>
       </c>
@@ -1174,7 +1174,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>56</v>
       </c>
@@ -1191,7 +1191,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>59</v>
       </c>
@@ -1208,7 +1208,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>62</v>
       </c>
@@ -1225,7 +1225,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>65</v>
       </c>
@@ -1242,7 +1242,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>68</v>
       </c>
@@ -1259,7 +1259,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>71</v>
       </c>
@@ -1276,7 +1276,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>74</v>
       </c>
@@ -1293,7 +1293,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>77</v>
       </c>
@@ -1310,7 +1310,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>79</v>
       </c>
@@ -1327,7 +1327,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>109</v>
       </c>
@@ -1344,7 +1344,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>112</v>
       </c>
@@ -1361,7 +1361,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="29" spans="1:5">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>113</v>
       </c>
@@ -1378,7 +1378,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>114</v>
       </c>
@@ -1395,7 +1395,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>115</v>
       </c>
@@ -1412,7 +1412,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>116</v>
       </c>
@@ -1429,7 +1429,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="33" spans="1:5">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>117</v>
       </c>
@@ -1446,7 +1446,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="34" spans="1:5">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>118</v>
       </c>
@@ -1463,7 +1463,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>119</v>
       </c>
@@ -1480,7 +1480,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>120</v>
       </c>
@@ -1497,7 +1497,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>121</v>
       </c>
@@ -1514,7 +1514,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>146</v>
       </c>
@@ -1531,7 +1531,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="39" spans="1:5">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>147</v>
       </c>
@@ -1548,7 +1548,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="40" spans="1:5">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>148</v>
       </c>
@@ -1565,7 +1565,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>149</v>
       </c>
@@ -1582,7 +1582,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>150</v>
       </c>
@@ -1599,7 +1599,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>122</v>
       </c>
@@ -1616,7 +1616,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>123</v>
       </c>
@@ -1633,7 +1633,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>124</v>
       </c>
@@ -1650,7 +1650,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="46" spans="1:5">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>125</v>
       </c>
@@ -1667,7 +1667,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="47" spans="1:5">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>126</v>
       </c>
@@ -1684,7 +1684,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>127</v>
       </c>
@@ -1701,7 +1701,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="49" spans="1:5">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>128</v>
       </c>
@@ -1718,7 +1718,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="50" spans="1:5">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>129</v>
       </c>
@@ -1735,7 +1735,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="51" spans="1:5">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>130</v>
       </c>
@@ -1752,7 +1752,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="52" spans="1:5">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>131</v>
       </c>
@@ -1769,7 +1769,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="53" spans="1:5">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>132</v>
       </c>
@@ -1786,7 +1786,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>133</v>
       </c>
@@ -1803,7 +1803,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="55" spans="1:5">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>134</v>
       </c>
@@ -1820,7 +1820,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="56" spans="1:5">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>135</v>
       </c>
@@ -1837,7 +1837,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="57" spans="1:5">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>136</v>
       </c>
@@ -1854,7 +1854,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="58" spans="1:5">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>137</v>
       </c>
@@ -1871,7 +1871,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="59" spans="1:5">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>138</v>
       </c>
@@ -1888,7 +1888,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="60" spans="1:5">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>139</v>
       </c>
@@ -1905,7 +1905,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="61" spans="1:5">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>140</v>
       </c>
@@ -1922,7 +1922,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="62" spans="1:5">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>141</v>
       </c>
@@ -1939,7 +1939,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="63" spans="1:5">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>142</v>
       </c>
@@ -1956,7 +1956,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="64" spans="1:5">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>143</v>
       </c>
@@ -1973,7 +1973,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="65" spans="1:5">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>144</v>
       </c>
@@ -1990,7 +1990,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="66" spans="1:5">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>145</v>
       </c>
@@ -2015,12 +2015,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -2031,7 +2031,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>8</v>
       </c>

</xml_diff>